<commit_message>
Lernmodul KI Aufg 3 mit Reiter
</commit_message>
<xml_diff>
--- a/faecher/informatik/klasse-9/1-Tabellenkalkulation/3-Funktionen.xlsx
+++ b/faecher/informatik/klasse-9/1-Tabellenkalkulation/3-Funktionen.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Inf_9\Tabellenkalkulation\01 Einführung + Funktionen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffran\Documents\git\unterricht\faecher\informatik\klasse-9\1-Tabellenkalkulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C43F0A-0E1D-4449-A5F8-F1F31BC6B465}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C43F0A-0E1D-4449-A5F8-F1F31BC6B465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Funktionen" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="152511" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -458,13 +458,11 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -479,7 +477,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -487,8 +484,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
@@ -901,1008 +896,978 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I66"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="1" max="1" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.26953125" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.7109375" customWidth="1"/>
-    <col min="5" max="5" width="39.42578125" customWidth="1"/>
+    <col min="4" max="4" width="1.7265625" customWidth="1"/>
+    <col min="5" max="5" width="39.453125" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
+    <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4" t="s">
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="2"/>
+      <c r="E4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="7">
         <v>39508</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>814.19</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="7" t="s">
+      <c r="D5" s="2"/>
+      <c r="E5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="5">
         <v>125</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="9">
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="7">
         <v>39509</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="7" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="5">
         <v>99</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="9">
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="7">
         <v>39510</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <v>378.32</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="7" t="s">
+      <c r="D7" s="2"/>
+      <c r="E7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="5">
         <v>52</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9">
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="7">
         <v>39511</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="8">
         <v>500.51</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="11" t="s">
+      <c r="D8" s="2"/>
+      <c r="E8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="9">
         <v>33</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9">
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="7">
         <v>39512</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="8">
         <v>678.78</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="12" t="s">
+      <c r="D9" s="2"/>
+      <c r="E9" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="37"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="40" t="s">
+      <c r="F9" s="32"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="I9" s="40"/>
-    </row>
-    <row r="10" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9">
+      <c r="I9" s="35"/>
+    </row>
+    <row r="10" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="7">
         <v>39513</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <v>920.13</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="12" t="s">
+      <c r="D10" s="2"/>
+      <c r="E10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="38"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9">
+      <c r="F10" s="33"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="7">
         <v>39514</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <v>809.23</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="12" t="s">
+      <c r="D11" s="2"/>
+      <c r="E11" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="39"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9">
+      <c r="F11" s="34"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="7">
         <v>39515</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <v>747.13</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="14" t="s">
+      <c r="D12" s="2"/>
+      <c r="E12" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9">
+      <c r="F12" s="34"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="7">
         <v>39516</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="12" t="s">
+      <c r="C13" s="8"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="39"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9">
+      <c r="F13" s="34"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="7">
         <v>39517</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <v>956.12</v>
       </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="16" t="s">
+      <c r="D14" s="2"/>
+      <c r="E14" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="37"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9">
+      <c r="F14" s="32"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="7">
         <v>39518</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="8">
         <v>515.21</v>
       </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="16" t="s">
+      <c r="D15" s="2"/>
+      <c r="E15" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="37"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9">
+      <c r="F15" s="32"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="7">
         <v>39519</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <v>780.51</v>
       </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-    </row>
-    <row r="17" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9">
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+    </row>
+    <row r="17" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="7">
         <v>39520</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <v>332.75</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="17" t="s">
+      <c r="D17" s="2"/>
+      <c r="E17" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="9">
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="7">
         <v>39521</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>982.24</v>
       </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="19" t="s">
+      <c r="D18" s="2"/>
+      <c r="E18" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-    </row>
-    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="9">
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="7">
         <v>39522</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <v>519.38</v>
       </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="7" t="s">
+      <c r="D19" s="2"/>
+      <c r="E19" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="9">
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="7">
         <v>39523</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="7" t="s">
+      <c r="C20" s="8"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="9">
+      <c r="F20" s="5"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="7">
         <v>39524</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="8">
         <v>741.1</v>
       </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="7" t="s">
+      <c r="D21" s="2"/>
+      <c r="E21" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-    </row>
-    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="9">
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="7">
         <v>39525</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C22" s="8">
         <v>500.82</v>
       </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="7" t="s">
+      <c r="D22" s="2"/>
+      <c r="E22" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F22" s="7"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="9">
+      <c r="F22" s="5"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="7">
         <v>39526</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="8">
         <v>326.16000000000003</v>
       </c>
-      <c r="D23" s="3"/>
-      <c r="E23" s="7" t="s">
+      <c r="D23" s="2"/>
+      <c r="E23" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-    </row>
-    <row r="24" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9">
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="7">
         <v>39527</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <v>663.77</v>
       </c>
-      <c r="D24" s="3"/>
-      <c r="E24" s="11" t="s">
+      <c r="D24" s="2"/>
+      <c r="E24" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-    </row>
-    <row r="25" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9">
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+    </row>
+    <row r="25" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="7">
         <v>39528</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="8">
         <v>596.61</v>
       </c>
-      <c r="D25" s="3"/>
-      <c r="E25" s="21" t="s">
+      <c r="D25" s="2"/>
+      <c r="E25" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="37"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9">
+      <c r="F25" s="32"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="7">
         <v>39529</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>733.19</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="21" t="s">
+      <c r="D26" s="2"/>
+      <c r="E26" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="F26" s="37"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-    </row>
-    <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="9">
+      <c r="F26" s="32"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="7">
         <v>39530</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="10"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="9">
+      <c r="C27" s="8"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="7">
         <v>39531</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="8">
         <v>983.17</v>
       </c>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="11" t="s">
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="9">
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="7">
         <v>39532</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="8">
         <v>888</v>
       </c>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="20" t="s">
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="9">
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="7">
         <v>39533</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="8">
         <v>943.61</v>
       </c>
-      <c r="D30" s="3"/>
-      <c r="E30" s="7" t="s">
+      <c r="D30" s="2"/>
+      <c r="E30" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="5">
         <v>3</v>
       </c>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="9">
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="7">
         <v>39534</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C31" s="8">
         <v>875.7</v>
       </c>
-      <c r="D31" s="3"/>
-      <c r="E31" s="7" t="s">
+      <c r="D31" s="2"/>
+      <c r="E31" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="5">
         <v>5</v>
       </c>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="9">
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="7">
         <v>39535</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="10">
+      <c r="C32" s="8">
         <v>411.92</v>
       </c>
-      <c r="D32" s="3"/>
-      <c r="E32" s="7" t="s">
+      <c r="D32" s="2"/>
+      <c r="E32" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-    </row>
-    <row r="33" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="9">
+      <c r="F32" s="5"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="7">
         <v>39536</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C33" s="10">
+      <c r="C33" s="8">
         <v>728.99</v>
       </c>
-      <c r="D33" s="3"/>
-      <c r="E33" s="7" t="s">
+      <c r="D33" s="2"/>
+      <c r="E33" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-    </row>
-    <row r="34" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="9">
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+    </row>
+    <row r="34" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="7">
         <v>39537</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C34" s="10"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="7" t="s">
+      <c r="C34" s="8"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="5">
         <v>5</v>
       </c>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-    </row>
-    <row r="35" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9">
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+    </row>
+    <row r="35" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="7">
         <v>39538</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="8">
         <v>375.65</v>
       </c>
-      <c r="D35" s="3"/>
-      <c r="E35" s="7" t="s">
+      <c r="D35" s="2"/>
+      <c r="E35" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F35" s="7">
+      <c r="F35" s="5">
         <v>4</v>
       </c>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-    </row>
-    <row r="36" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="17" t="s">
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+    </row>
+    <row r="36" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="27"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="11" t="s">
+      <c r="B36" s="22"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F36" s="11" t="s">
+      <c r="F36" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-    </row>
-    <row r="37" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="17" t="s">
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+    </row>
+    <row r="37" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B37" s="27"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="21" t="s">
+      <c r="B37" s="22"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="F37" s="37"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-    </row>
-    <row r="38" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="17" t="s">
+      <c r="F37" s="32"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+    </row>
+    <row r="38" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="21" t="s">
+      <c r="B38" s="22"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="F38" s="37"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-    </row>
-    <row r="39" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="22" t="s">
+      <c r="F38" s="32"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+    </row>
+    <row r="39" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="28"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="21" t="s">
+      <c r="B39" s="23"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F39" s="37"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5"/>
-      <c r="J39" s="2"/>
-    </row>
-    <row r="40" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="17" t="s">
+      <c r="F39" s="32"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+    </row>
+    <row r="40" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="2"/>
-    </row>
-    <row r="41" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="17" t="s">
+      <c r="B40" s="22"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+    </row>
+    <row r="41" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B41" s="27"/>
-      <c r="C41" s="33"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="2"/>
-    </row>
-    <row r="42" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="17" t="s">
+      <c r="B41" s="22"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+    </row>
+    <row r="42" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B42" s="27"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="2"/>
-    </row>
-    <row r="43" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="14" t="s">
+      <c r="B42" s="22"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+    </row>
+    <row r="43" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B43" s="29"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-      <c r="I43" s="5"/>
-      <c r="J43" s="2"/>
-    </row>
-    <row r="44" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="17" t="s">
+      <c r="B43" s="24"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+    </row>
+    <row r="44" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="27"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5"/>
-      <c r="J44" s="2"/>
-    </row>
-    <row r="45" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="17" t="s">
+      <c r="B44" s="22"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+    </row>
+    <row r="45" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B45" s="27"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="2"/>
-    </row>
-    <row r="46" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="14" t="s">
+      <c r="B45" s="22"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+    </row>
+    <row r="46" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B46" s="29"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="23"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="5"/>
-      <c r="J46" s="2"/>
-    </row>
-    <row r="47" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="17" t="s">
+      <c r="B46" s="24"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+    </row>
+    <row r="47" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A47" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="27"/>
-      <c r="C47" s="35"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="23"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
-      <c r="I47" s="5"/>
-      <c r="J47" s="2"/>
-    </row>
-    <row r="48" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="22" t="s">
+      <c r="B47" s="22"/>
+      <c r="C47" s="30"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+    </row>
+    <row r="48" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A48" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B48" s="28"/>
-      <c r="C48" s="36"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="23"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
-      <c r="I48" s="5"/>
-      <c r="J48" s="2"/>
-    </row>
-    <row r="49" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="17" t="s">
+      <c r="B48" s="23"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+    </row>
+    <row r="49" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A49" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B49" s="27"/>
-      <c r="C49" s="35"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="24"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="25"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="2"/>
-    </row>
-    <row r="50" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="17" t="s">
+      <c r="B49" s="22"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="11"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+    </row>
+    <row r="50" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A50" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="27"/>
-      <c r="C50" s="31"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="24"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="25"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="5"/>
-      <c r="J50" s="2"/>
-    </row>
-    <row r="51" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="24"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="25"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="2"/>
-    </row>
-    <row r="52" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="24"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="24"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="25"/>
-      <c r="H52" s="5"/>
-      <c r="I52" s="5"/>
-      <c r="J52" s="2"/>
-    </row>
-    <row r="53" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="24"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="26"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="24"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="25"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5"/>
-      <c r="J53" s="2"/>
-    </row>
-    <row r="54" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="24"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="24"/>
-      <c r="F54" s="26"/>
-      <c r="G54" s="25"/>
-      <c r="H54" s="5"/>
-      <c r="I54" s="5"/>
-      <c r="J54" s="2"/>
-    </row>
-    <row r="55" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" s="24"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="24"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="25"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-      <c r="J55" s="2"/>
-    </row>
-    <row r="56" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="24"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="26"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="5"/>
-      <c r="I56" s="5"/>
-      <c r="J56" s="2"/>
-    </row>
-    <row r="57" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="24"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5"/>
-      <c r="J57" s="2"/>
-    </row>
-    <row r="58" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A58" s="24"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
-      <c r="H58" s="5"/>
-      <c r="I58" s="5"/>
-      <c r="J58" s="2"/>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B50" s="22"/>
+      <c r="C50" s="26"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+    </row>
+    <row r="51" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+    </row>
+    <row r="52" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+    </row>
+    <row r="53" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+    </row>
+    <row r="54" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="21"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="21"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+    </row>
+    <row r="55" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+    </row>
+    <row r="56" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="21"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+    </row>
+    <row r="57" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+    </row>
+    <row r="58" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
     </row>
   </sheetData>

</xml_diff>